<commit_message>
Added Curie temperature processing scripts and kappabridge data.
</commit_message>
<xml_diff>
--- a/data/raw/metadata.xlsx
+++ b/data/raw/metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paselkin\Dropbox\Research\Glaciers2Bay\glacier-bay-uwt-student-projects\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1BCD19-8D2A-4D25-A1E7-1CD4ED65E6D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8933E0-A0AB-4EFF-B69F-F2268104DCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,11 +16,16 @@
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="188">
   <si>
     <t>2022CB0101.irmdcd</t>
   </si>
@@ -563,6 +568,27 @@
   </si>
   <si>
     <t>2022EG0103.hysu</t>
+  </si>
+  <si>
+    <t>curie_file</t>
+  </si>
+  <si>
+    <t>24PR20C.CUR</t>
+  </si>
+  <si>
+    <t>24WR20C.CUR</t>
+  </si>
+  <si>
+    <t>24WR21.CUR</t>
+  </si>
+  <si>
+    <t>25GP01A1.CUR</t>
+  </si>
+  <si>
+    <t>25MM10A2.CUR</t>
+  </si>
+  <si>
+    <t>25MM11A1.CUR</t>
   </si>
 </sst>
 </file>
@@ -1407,19 +1433,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="27.53125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.53125" customWidth="1"/>
-    <col min="3" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.73046875" customWidth="1"/>
-    <col min="12" max="12" width="9.06640625" style="1"/>
+    <col min="2" max="3" width="27.53125" customWidth="1"/>
+    <col min="4" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.73046875" customWidth="1"/>
+    <col min="13" max="13" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>96</v>
       </c>
@@ -1427,479 +1453,482 @@
         <v>132</v>
       </c>
       <c r="C1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>42</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>43</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>53</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>163</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>44</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>133</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>33</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>99</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2022</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>51</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>50</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="1">
         <v>0.29509998999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>134</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>39</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>99</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>2022</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>51</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>50</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="1">
         <v>0.28129999</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>135</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>46</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>47</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>100</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>48</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>2022</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>49</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>54</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="1">
         <v>0.37259998999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>180</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>35</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>47</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>100</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>48</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>2022</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>49</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>54</v>
       </c>
-      <c r="L5" s="1">
+      <c r="M5" s="1">
         <v>0.28129999</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>180</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>47</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>100</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>48</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>2022</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>49</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>54</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="1">
         <v>0.28129999</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>136</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>52</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>100</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>48</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>2022</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>49</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>54</v>
       </c>
-      <c r="L7" s="1">
+      <c r="M7" s="1">
         <v>0.34410000000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>137</v>
       </c>
-      <c r="C8" t="s">
-        <v>70</v>
-      </c>
       <c r="D8" t="s">
         <v>70</v>
       </c>
       <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
         <v>101</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>2023</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>71</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="1">
+      <c r="M8" s="1">
         <v>0.22339999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>7</v>
       </c>
       <c r="B9" t="s">
         <v>138</v>
       </c>
-      <c r="C9" t="s">
-        <v>75</v>
-      </c>
       <c r="D9" t="s">
         <v>75</v>
       </c>
       <c r="E9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" t="s">
         <v>101</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>2023</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>72</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>73</v>
       </c>
-      <c r="K9" t="s">
-        <v>74</v>
-      </c>
-      <c r="L9" s="1">
+      <c r="L9" t="s">
+        <v>74</v>
+      </c>
+      <c r="M9" s="1">
         <v>0.10970000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>8</v>
       </c>
       <c r="B10" t="s">
         <v>139</v>
       </c>
-      <c r="C10" t="s">
-        <v>76</v>
-      </c>
       <c r="D10" t="s">
         <v>76</v>
       </c>
       <c r="E10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
         <v>102</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>2023</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>71</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>73</v>
       </c>
-      <c r="L10" s="1">
+      <c r="M10" s="1">
         <v>0.2767</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>9</v>
       </c>
       <c r="B11" t="s">
         <v>140</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>77</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>55</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>103</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>106</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>2025</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>72</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>107</v>
       </c>
-      <c r="K11" t="s">
-        <v>74</v>
-      </c>
-      <c r="L11" s="1">
+      <c r="L11" t="s">
+        <v>74</v>
+      </c>
+      <c r="M11" s="1">
         <v>4.3799999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12" t="s">
         <v>141</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>78</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>56</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>104</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>97</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>124</v>
       </c>
-      <c r="K12" t="s">
-        <v>74</v>
-      </c>
-      <c r="L12" s="1">
+      <c r="L12" t="s">
+        <v>74</v>
+      </c>
+      <c r="M12" s="1">
         <v>0.1018</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13" t="s">
         <v>142</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>79</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>87</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>105</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>97</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>124</v>
       </c>
-      <c r="K13" t="s">
-        <v>74</v>
-      </c>
-      <c r="L13" s="1">
+      <c r="L13" t="s">
+        <v>74</v>
+      </c>
+      <c r="M13" s="1">
         <v>0.1198</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14" t="s">
         <v>143</v>
       </c>
-      <c r="C14" t="s">
-        <v>57</v>
-      </c>
       <c r="D14" t="s">
         <v>57</v>
       </c>
       <c r="E14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" t="s">
         <v>101</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>48</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>2024</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>72</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>73</v>
       </c>
-      <c r="K14" t="s">
-        <v>74</v>
-      </c>
-      <c r="L14" s="1">
+      <c r="L14" t="s">
+        <v>74</v>
+      </c>
+      <c r="M14" s="1">
         <v>3.1E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>13</v>
       </c>
       <c r="B15" t="s">
         <v>144</v>
       </c>
-      <c r="C15" t="s">
-        <v>58</v>
-      </c>
       <c r="D15" t="s">
         <v>58</v>
       </c>
       <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
         <v>101</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>48</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>2024</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>71</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>73</v>
       </c>
-      <c r="K15" t="s">
-        <v>74</v>
-      </c>
-      <c r="L15" s="1">
+      <c r="L15" t="s">
+        <v>74</v>
+      </c>
+      <c r="M15" s="1">
         <v>0.1255</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1907,314 +1936,317 @@
         <v>145</v>
       </c>
       <c r="C16" t="s">
+        <v>182</v>
+      </c>
+      <c r="D16" t="s">
         <v>80</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>59</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>102</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>106</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <v>2025</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>72</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>73</v>
       </c>
-      <c r="K16" t="s">
-        <v>74</v>
-      </c>
-      <c r="L16" s="1">
+      <c r="L16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M16" s="1">
         <v>0.1182</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>146</v>
       </c>
-      <c r="C17" t="s">
-        <v>60</v>
-      </c>
       <c r="D17" t="s">
         <v>60</v>
       </c>
       <c r="E17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" t="s">
         <v>102</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>106</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <v>2025</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>71</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>73</v>
       </c>
-      <c r="K17" t="s">
-        <v>74</v>
-      </c>
-      <c r="L17" s="1">
+      <c r="L17" t="s">
+        <v>74</v>
+      </c>
+      <c r="M17" s="1">
         <v>0.11</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>16</v>
       </c>
       <c r="B18" t="s">
         <v>147</v>
       </c>
-      <c r="C18" t="s">
-        <v>61</v>
-      </c>
       <c r="D18" t="s">
         <v>61</v>
       </c>
       <c r="E18" t="s">
+        <v>61</v>
+      </c>
+      <c r="F18" t="s">
         <v>108</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>106</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <v>2025</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>71</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>73</v>
       </c>
-      <c r="K18" t="s">
-        <v>74</v>
-      </c>
-      <c r="L18" s="1">
+      <c r="L18" t="s">
+        <v>74</v>
+      </c>
+      <c r="M18" s="1">
         <v>3.4700000000000002E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>148</v>
       </c>
-      <c r="C19" t="s">
-        <v>62</v>
-      </c>
       <c r="D19" t="s">
         <v>62</v>
       </c>
       <c r="E19" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" t="s">
         <v>109</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>106</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <v>2024</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>71</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>125</v>
       </c>
-      <c r="K19" t="s">
-        <v>74</v>
-      </c>
-      <c r="L19" s="1">
+      <c r="L19" t="s">
+        <v>74</v>
+      </c>
+      <c r="M19" s="1">
         <v>5.3199999999999997E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>149</v>
       </c>
-      <c r="C20" t="s">
-        <v>63</v>
-      </c>
       <c r="D20" t="s">
         <v>63</v>
       </c>
       <c r="E20" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" t="s">
         <v>109</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>48</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <v>2024</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>71</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>125</v>
       </c>
-      <c r="K20" t="s">
-        <v>74</v>
-      </c>
-      <c r="L20" s="1">
+      <c r="L20" t="s">
+        <v>74</v>
+      </c>
+      <c r="M20" s="1">
         <v>7.7600000000000002E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>150</v>
       </c>
-      <c r="C21" t="s">
-        <v>64</v>
-      </c>
       <c r="D21" t="s">
         <v>64</v>
       </c>
       <c r="E21" t="s">
+        <v>64</v>
+      </c>
+      <c r="F21" t="s">
         <v>109</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>106</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>2025</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>71</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>125</v>
       </c>
-      <c r="K21" t="s">
-        <v>74</v>
-      </c>
-      <c r="L21" s="1">
+      <c r="L21" t="s">
+        <v>74</v>
+      </c>
+      <c r="M21" s="1">
         <v>4.4900000000000002E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>151</v>
       </c>
-      <c r="C22" t="s">
-        <v>65</v>
-      </c>
       <c r="D22" t="s">
         <v>65</v>
       </c>
       <c r="E22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" t="s">
         <v>110</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>106</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>2024</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>71</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>54</v>
       </c>
-      <c r="K22" t="s">
-        <v>74</v>
-      </c>
-      <c r="L22" s="1">
+      <c r="L22" t="s">
+        <v>74</v>
+      </c>
+      <c r="M22" s="1">
         <v>8.2100000000000006E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>152</v>
       </c>
-      <c r="C23" t="s">
-        <v>66</v>
-      </c>
       <c r="D23" t="s">
         <v>66</v>
       </c>
       <c r="E23" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" t="s">
         <v>110</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>48</v>
       </c>
-      <c r="G23">
+      <c r="H23">
         <v>2024</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>72</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>54</v>
       </c>
-      <c r="K23" t="s">
-        <v>74</v>
-      </c>
-      <c r="L23" s="1">
+      <c r="L23" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="1">
         <v>1.46E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>153</v>
       </c>
-      <c r="C24" t="s">
-        <v>67</v>
-      </c>
       <c r="D24" t="s">
         <v>67</v>
       </c>
       <c r="E24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24" t="s">
         <v>110</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>48</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>2024</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>71</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>54</v>
       </c>
-      <c r="K24" t="s">
-        <v>74</v>
-      </c>
-      <c r="L24" s="1">
+      <c r="L24" t="s">
+        <v>74</v>
+      </c>
+      <c r="M24" s="1">
         <v>7.3899999999999993E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -2222,34 +2254,37 @@
         <v>154</v>
       </c>
       <c r="C25" t="s">
+        <v>183</v>
+      </c>
+      <c r="D25" t="s">
         <v>81</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>68</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>110</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>106</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>2025</v>
       </c>
-      <c r="H25" t="s">
+      <c r="I25" t="s">
         <v>72</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>54</v>
       </c>
-      <c r="K25" t="s">
-        <v>74</v>
-      </c>
-      <c r="L25" s="1">
+      <c r="L25" t="s">
+        <v>74</v>
+      </c>
+      <c r="M25" s="1">
         <v>0.1026</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -2257,130 +2292,133 @@
         <v>155</v>
       </c>
       <c r="C26" t="s">
-        <v>69</v>
+        <v>184</v>
       </c>
       <c r="D26" t="s">
         <v>69</v>
       </c>
       <c r="E26" t="s">
+        <v>69</v>
+      </c>
+      <c r="F26" t="s">
         <v>110</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>106</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>2025</v>
       </c>
-      <c r="H26" t="s">
+      <c r="I26" t="s">
         <v>71</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>54</v>
       </c>
-      <c r="K26" t="s">
-        <v>74</v>
-      </c>
-      <c r="L26" s="1">
+      <c r="L26" t="s">
+        <v>74</v>
+      </c>
+      <c r="M26" s="1">
         <v>0.15029999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>166</v>
       </c>
       <c r="B27" t="s">
         <v>167</v>
       </c>
-      <c r="C27" t="s">
-        <v>168</v>
-      </c>
       <c r="D27" t="s">
         <v>168</v>
       </c>
       <c r="E27" t="s">
+        <v>168</v>
+      </c>
+      <c r="F27" t="s">
         <v>120</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>48</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>49</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>107</v>
       </c>
-      <c r="K27" t="s">
-        <v>74</v>
-      </c>
-      <c r="L27" s="1">
+      <c r="L27" t="s">
+        <v>74</v>
+      </c>
+      <c r="M27" s="1">
         <v>9.8400000000000001E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>169</v>
       </c>
       <c r="B28" t="s">
         <v>170</v>
       </c>
-      <c r="C28" t="s">
-        <v>171</v>
-      </c>
       <c r="D28" t="s">
         <v>171</v>
       </c>
       <c r="E28" t="s">
+        <v>171</v>
+      </c>
+      <c r="F28" t="s">
         <v>120</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>48</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
         <v>49</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>107</v>
       </c>
-      <c r="K28" t="s">
-        <v>74</v>
-      </c>
-      <c r="L28" s="1">
+      <c r="L28" t="s">
+        <v>74</v>
+      </c>
+      <c r="M28" s="1">
         <v>8.9700000000000002E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>172</v>
       </c>
       <c r="B29" t="s">
         <v>173</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>174</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>175</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F29" t="s">
         <v>120</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>48</v>
       </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>49</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>107</v>
       </c>
-      <c r="K29" t="s">
-        <v>74</v>
-      </c>
-      <c r="L29" s="1">
+      <c r="L29" t="s">
+        <v>74</v>
+      </c>
+      <c r="M29" s="1">
         <v>4.0300000000000002E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -2388,63 +2426,66 @@
         <v>156</v>
       </c>
       <c r="C30" t="s">
+        <v>185</v>
+      </c>
+      <c r="D30" t="s">
         <v>82</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>88</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>121</v>
       </c>
-      <c r="H30" t="s">
+      <c r="I30" t="s">
         <v>97</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>128</v>
       </c>
-      <c r="K30" t="s">
-        <v>74</v>
-      </c>
-      <c r="L30" s="1">
+      <c r="L30" t="s">
+        <v>74</v>
+      </c>
+      <c r="M30" s="1">
         <v>0.123</v>
       </c>
-      <c r="M30" t="s">
+      <c r="N30" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>26</v>
       </c>
       <c r="B31" t="s">
         <v>157</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>83</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>89</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>121</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
         <v>97</v>
       </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>127</v>
       </c>
-      <c r="K31" t="s">
-        <v>74</v>
-      </c>
-      <c r="L31" s="1">
+      <c r="L31" t="s">
+        <v>74</v>
+      </c>
+      <c r="M31" s="1">
         <v>0.1333</v>
       </c>
-      <c r="M31" t="s">
+      <c r="N31" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -2452,28 +2493,31 @@
         <v>158</v>
       </c>
       <c r="C32" t="s">
+        <v>186</v>
+      </c>
+      <c r="D32" t="s">
         <v>85</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>90</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>122</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>97</v>
       </c>
-      <c r="J32" t="s">
+      <c r="K32" t="s">
         <v>124</v>
       </c>
-      <c r="K32" t="s">
-        <v>74</v>
-      </c>
-      <c r="L32" s="1">
+      <c r="L32" t="s">
+        <v>74</v>
+      </c>
+      <c r="M32" s="1">
         <v>0.1096</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -2481,283 +2525,286 @@
         <v>159</v>
       </c>
       <c r="C33" t="s">
+        <v>187</v>
+      </c>
+      <c r="D33" t="s">
         <v>86</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>91</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>123</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>97</v>
       </c>
-      <c r="J33" t="s">
+      <c r="K33" t="s">
         <v>124</v>
       </c>
-      <c r="K33" t="s">
-        <v>74</v>
-      </c>
-      <c r="L33" s="1">
+      <c r="L33" t="s">
+        <v>74</v>
+      </c>
+      <c r="M33" s="1">
         <v>0.1376</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>29</v>
       </c>
       <c r="B34" t="s">
         <v>160</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>84</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
         <v>92</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>164</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>97</v>
       </c>
-      <c r="J34" t="s">
+      <c r="K34" t="s">
         <v>126</v>
       </c>
-      <c r="K34" t="s">
-        <v>74</v>
-      </c>
-      <c r="L34" s="1">
+      <c r="L34" t="s">
+        <v>74</v>
+      </c>
+      <c r="M34" s="1">
         <v>0.13489999999999999</v>
       </c>
-      <c r="M34" t="s">
+      <c r="N34" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>30</v>
       </c>
       <c r="B35" t="s">
         <v>161</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>94</v>
       </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>93</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>165</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>97</v>
       </c>
-      <c r="J35" t="s">
+      <c r="K35" t="s">
         <v>127</v>
       </c>
-      <c r="K35" t="s">
-        <v>74</v>
-      </c>
-      <c r="L35" s="1">
+      <c r="L35" t="s">
+        <v>74</v>
+      </c>
+      <c r="M35" s="1">
         <v>0.10829999999999999</v>
       </c>
-      <c r="M35" t="s">
+      <c r="N35" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>111</v>
       </c>
       <c r="B36" t="s">
         <v>176</v>
       </c>
-      <c r="C36" t="s">
-        <v>112</v>
-      </c>
       <c r="D36" t="s">
         <v>112</v>
       </c>
       <c r="E36" t="s">
+        <v>112</v>
+      </c>
+      <c r="F36" t="s">
         <v>101</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>106</v>
       </c>
-      <c r="G36">
+      <c r="H36">
         <v>2024</v>
       </c>
-      <c r="H36" t="s">
+      <c r="I36" t="s">
         <v>71</v>
       </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>73</v>
       </c>
-      <c r="K36" t="s">
-        <v>74</v>
-      </c>
-      <c r="L36" s="1">
+      <c r="L36" t="s">
+        <v>74</v>
+      </c>
+      <c r="M36" s="1">
         <v>4.7600000000000003E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>113</v>
       </c>
       <c r="B37" t="s">
         <v>177</v>
       </c>
-      <c r="C37" t="s">
-        <v>114</v>
-      </c>
       <c r="D37" t="s">
         <v>114</v>
       </c>
       <c r="E37" t="s">
+        <v>114</v>
+      </c>
+      <c r="F37" t="s">
         <v>102</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>106</v>
       </c>
-      <c r="G37">
+      <c r="H37">
         <v>2024</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>71</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
         <v>73</v>
       </c>
-      <c r="K37" t="s">
-        <v>74</v>
-      </c>
-      <c r="L37" s="1">
+      <c r="L37" t="s">
+        <v>74</v>
+      </c>
+      <c r="M37" s="1">
         <v>1.54E-2</v>
       </c>
-      <c r="M37" t="s">
+      <c r="N37" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>115</v>
       </c>
       <c r="B38" t="s">
         <v>178</v>
       </c>
-      <c r="C38" t="s">
-        <v>116</v>
-      </c>
       <c r="D38" t="s">
         <v>116</v>
       </c>
       <c r="E38" t="s">
+        <v>116</v>
+      </c>
+      <c r="F38" t="s">
         <v>102</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>48</v>
       </c>
-      <c r="G38">
+      <c r="H38">
         <v>2024</v>
       </c>
-      <c r="H38" t="s">
+      <c r="I38" t="s">
         <v>72</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>73</v>
       </c>
-      <c r="K38" t="s">
-        <v>74</v>
-      </c>
-      <c r="L38" s="1">
+      <c r="L38" t="s">
+        <v>74</v>
+      </c>
+      <c r="M38" s="1">
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>117</v>
       </c>
       <c r="B39" t="s">
         <v>179</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>118</v>
       </c>
-      <c r="D39" t="s">
+      <c r="E39" t="s">
         <v>119</v>
       </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
         <v>108</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>106</v>
       </c>
-      <c r="G39">
+      <c r="H39">
         <v>2025</v>
       </c>
-      <c r="H39" t="s">
+      <c r="I39" t="s">
         <v>72</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>73</v>
       </c>
-      <c r="K39" t="s">
-        <v>74</v>
-      </c>
-      <c r="L39" s="1">
+      <c r="L39" t="s">
+        <v>74</v>
+      </c>
+      <c r="M39" s="1">
         <v>2.92E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>31</v>
       </c>
       <c r="B40" t="s">
         <v>162</v>
       </c>
-      <c r="C40" t="s">
-        <v>95</v>
-      </c>
       <c r="D40" t="s">
         <v>95</v>
       </c>
       <c r="E40" t="s">
+        <v>95</v>
+      </c>
+      <c r="F40" t="s">
         <v>98</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>51</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>50</v>
       </c>
-      <c r="L40" s="1">
+      <c r="M40" s="1">
         <v>0.27910000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>32</v>
       </c>
       <c r="B41" t="s">
         <v>162</v>
       </c>
-      <c r="C41" t="s">
-        <v>95</v>
-      </c>
       <c r="D41" t="s">
         <v>95</v>
       </c>
       <c r="E41" t="s">
+        <v>95</v>
+      </c>
+      <c r="F41" t="s">
         <v>98</v>
       </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>51</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>50</v>
       </c>
-      <c r="L41" s="1">
+      <c r="M41" s="1">
         <v>0.27910000000000001</v>
       </c>
     </row>

</xml_diff>